<commit_message>
new update existing bulk import
</commit_message>
<xml_diff>
--- a/scripts/demo-import-test.xlsx
+++ b/scripts/demo-import-test.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:T5"/>
+  <dimension ref="A1:V5"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -458,6 +458,12 @@
         <v>continuity_last_verified</v>
       </c>
       <c r="T1" t="str">
+        <v>continuity_history</v>
+      </c>
+      <c r="U1" t="str">
+        <v>revalidation_history</v>
+      </c>
+      <c r="V1" t="str">
         <v>revalidation_method</v>
       </c>
     </row>
@@ -520,6 +526,12 @@
         <v>2025-12-01</v>
       </c>
       <c r="T2" t="str">
+        <v>2019-12-01;2020-06-01;2021-06-01;2023-06-01;2025-12-01</v>
+      </c>
+      <c r="U2" t="str">
+        <v>2021-06-10;2023-06-10</v>
+      </c>
+      <c r="V2" t="str">
         <v>9.3a</v>
       </c>
     </row>
@@ -582,6 +594,12 @@
         <v>2026-01-10</v>
       </c>
       <c r="T3" t="str">
+        <v>2025-05-15;2025-11-15;2026-01-10</v>
+      </c>
+      <c r="U3" t="str">
+        <v/>
+      </c>
+      <c r="V3" t="str">
         <v>9.3b</v>
       </c>
     </row>
@@ -644,6 +662,12 @@
         <v/>
       </c>
       <c r="T4" t="str">
+        <v/>
+      </c>
+      <c r="U4" t="str">
+        <v/>
+      </c>
+      <c r="V4" t="str">
         <v>9.3b</v>
       </c>
     </row>
@@ -708,10 +732,16 @@
       <c r="T5" t="str">
         <v/>
       </c>
+      <c r="U5" t="str">
+        <v/>
+      </c>
+      <c r="V5" t="str">
+        <v/>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:T5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:V5"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>